<commit_message>
E2E fixture: tekrarlanan iki ürün kodu ayrıştırıldı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pTZGcw8vUPucFnSucXbLy
</commit_message>
<xml_diff>
--- a/procurement-platform/e2e/fixtures/01-stok-500-urun.xlsx
+++ b/procurement-platform/e2e/fixtures/01-stok-500-urun.xlsx
@@ -6046,7 +6046,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>KMP-25KVAR-400V-ADET</t>
+          <t>KMP-25KVAR-400V-ADET-2</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>KMP-25KVAR-440V-ADET</t>
+          <t>KMP-25KVAR-440V-ADET-2</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">

</xml_diff>